<commit_message>
Update content log: S-fold measure guide entry
</commit_message>
<xml_diff>
--- a/content-log.xlsx
+++ b/content-log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,6 +487,48 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>75eec08</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Measure Guide</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>How to Measure for S-Fold Curtains</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>guides/measure/s-fold-curtains.html</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://cpccai97-source.github.io/iseekblinds/guides/measure/s-fold-curtains.html</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>how to measure s-fold curtains, s-fold curtain measurement guide, wave curtains measuring</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>S-Fold Curtains</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Published</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log S-fold curtains install guide in content-log.xlsx
</commit_message>
<xml_diff>
--- a/content-log.xlsx
+++ b/content-log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,6 +529,43 @@
       <c r="H3" t="inlineStr">
         <is>
           <t>Published</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Install Guide</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>How to Install S-Fold Curtains</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://cpccai97-source.github.io/iseekblinds/guides/install/s-fold-curtains.html</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>how to install s-fold curtains, s-fold curtain installation, wave curtain track installation, ceiling mount s-fold track, s-fold gliders spacing</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>S-Fold Curtains / Curtain Tracks</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>5001df7</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log: vertical blinds complete guide
</commit_message>
<xml_diff>
--- a/content-log.xlsx
+++ b/content-log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -566,6 +566,43 @@
       <c r="G4" t="inlineStr">
         <is>
           <t>5001df7</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Vertical Blinds Complete Guide</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://cpccai97-source.github.io/iseekblinds/guides/vertical-blinds-complete-guide.html</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>vertical blinds Melbourne, PVC vertical blinds, fabric vertical blinds, vertical blinds sliding doors, vertical blinds cost Melbourne</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Vertical Blinds, Sliding Doors</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>f0662a1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-log: sheer curtains complete guide
</commit_message>
<xml_diff>
--- a/content-log.xlsx
+++ b/content-log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -603,6 +603,48 @@
       <c r="G5" t="inlineStr">
         <is>
           <t>f0662a1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Sheer Curtains — Complete Guide</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>guides/sheer-curtains-complete-guide.html</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>sheer curtains Melbourne, voile curtains, linen sheer curtains, sheer curtains privacy, sheer curtains with blinds, custom sheer curtains</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Sheer Curtains, Custom Curtains Melbourne</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>4e78e3f</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Published</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
log: content-log.xlsx entry for allergy guide
</commit_message>
<xml_diff>
--- a/content-log.xlsx
+++ b/content-log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -643,6 +643,48 @@
         </is>
       </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Best Blinds for Allergy &amp; Asthma Sufferers</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>guides/allergy-asthma-friendly-blinds.html</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>hypoallergenic blinds Melbourne, blinds for allergy sufferers Australia, dust free blinds, asthma friendly window treatments</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>All Products</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>40d76fa</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>Published</t>
         </is>

</xml_diff>

<commit_message>
log: record bifold door blinds blog post
</commit_message>
<xml_diff>
--- a/content-log.xlsx
+++ b/content-log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -685,6 +685,48 @@
         </is>
       </c>
       <c r="H7" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Bifold Door Blinds: 6 Solutions That Actually Work</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://cpccai97-source.github.io/iseekblinds/blog/bifold-door-blinds-solutions.html</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>bifold door blinds, blinds for bifold doors, panel glide blinds bifold, vertical blinds bifold doors</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Panel Glide, Vertical Blinds, Roller Blinds, Motorised Blinds</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>9f79a6b</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>Published</t>
         </is>

</xml_diff>

<commit_message>
Update content-log: motorised vs manual blinds guide
</commit_message>
<xml_diff>
--- a/content-log.xlsx
+++ b/content-log.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +48,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -732,6 +735,46 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>46100</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Motorised vs Manual Blinds: Which Is Right for Your Home?</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>guides/motorised-vs-manual-blinds.html</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>motorised blinds, manual blinds, motorised vs manual blinds, smart blinds australia, electric blinds melbourne</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Motorised blinds, manual blinds, roller blinds, honeycomb blinds</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>af7b0ca</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Log: woven wood measure guide in content-log.xlsx
</commit_message>
<xml_diff>
--- a/content-log.xlsx
+++ b/content-log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -775,6 +775,48 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Guide</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>How to Measure for Woven Wood &amp; Bamboo Blinds</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>guides/measure/woven-wood-blinds.html</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>how to measure woven wood blinds, bamboo blind measurement guide, natural blind inside mount, woven wood blinds Melbourne</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Woven wood blinds, bamboo blinds, natural blinds</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>011675a</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
blog: Garage Blinds Options Australia (garage blinds, PVC roller, venetian, buying guide)
</commit_message>
<xml_diff>
--- a/content-log.xlsx
+++ b/content-log.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -817,6 +817,75 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Guide - Install</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>How to Install Woven Wood &amp; Bamboo Blinds</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://cpccai97-source.github.io/iseekblinds/guides/install/woven-wood-blinds.html</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>how to install woven wood blinds, bamboo blind installation, natural blind DIY install, woven wood brackets Australia</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>5359433</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Guide (Complete)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Plantation Shutters Complete Guide — Timber, PVC &amp; Aluminium</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://cpccai97-source.github.io/iseekblinds/guides/plantation-shutters-complete-guide.html</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>plantation shutters Melbourne, plantation shutters guide, timber plantation shutters, PVC plantation shutters, plantation shutters cost Melbourne</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Plantation Shutters</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>c307eb6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>